<commit_message>
Update wifi sizing script
</commit_message>
<xml_diff>
--- a/Wi-Fi/Wi-Fi_Sizing_Script_8.1.xlsx
+++ b/Wi-Fi/Wi-Fi_Sizing_Script_8.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sainamithanagireddy/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CE2F1B-6D21-CD4B-81BE-F6A0F33467AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2190D5C-8792-DE43-BF31-985D27ACE6A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29920" windowHeight="17000" firstSheet="1" activeTab="1" xr2:uid="{CD935837-EFB7-7640-805F-6441372B141E}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29920" windowHeight="17000" firstSheet="1" activeTab="2" xr2:uid="{CD935837-EFB7-7640-805F-6441372B141E}"/>
   </bookViews>
   <sheets>
     <sheet name="PAS sizing" sheetId="3" r:id="rId1"/>
@@ -621,6 +621,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -628,12 +629,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -641,6 +644,7 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2135,7 +2139,7 @@
       </c>
       <c r="C6" s="23">
         <f xml:space="preserve"> (C62 * F10) + (C70 * F11) + (C74 * F14)</f>
-        <v>10673</v>
+        <v>3196</v>
       </c>
       <c r="D6" s="20"/>
       <c r="E6" s="20"/>
@@ -2148,7 +2152,7 @@
       </c>
       <c r="C7" s="24">
         <f xml:space="preserve"> (C62 * F10)/F18 + (C70 * F11)/F18 + (C74 * F14)/F18</f>
-        <v>35.576666666666668</v>
+        <v>10.653333333333334</v>
       </c>
       <c r="D7" s="20"/>
       <c r="E7" s="20"/>
@@ -2947,8 +2951,8 @@
         <v>159</v>
       </c>
       <c r="C62" s="21">
-        <f>SUMPRODUCT(C10:C31, F18:F39)+SUM(C32:C60)</f>
-        <v>10364</v>
+        <f>SUMPRODUCT(C10:C31, F21:F42)+SUM(C32:C60)</f>
+        <v>2887</v>
       </c>
       <c r="D62" s="20"/>
       <c r="E62" s="20"/>

</xml_diff>